<commit_message>
corregí calculos de show na, dataset emprolijado
</commit_message>
<xml_diff>
--- a/Reporte_Estructura_Dataset.xlsx
+++ b/Reporte_Estructura_Dataset.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="244">
   <si>
     <t>Grupo</t>
   </si>
@@ -94,9 +94,6 @@
     <t>avg_venue_capacity_total</t>
   </si>
   <si>
-    <t>has_live_data</t>
-  </si>
-  <si>
     <t>main_currency_2024</t>
   </si>
   <si>
@@ -148,12 +145,6 @@
     <t>n_shows_with_capacity_total</t>
   </si>
   <si>
-    <t>off_cycle</t>
-  </si>
-  <si>
-    <t>shows_2026</t>
-  </si>
-  <si>
     <t>shows_per_country_2024</t>
   </si>
   <si>
@@ -331,16 +322,19 @@
     <t>float64</t>
   </si>
   <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>Int64</t>
+  </si>
+  <si>
     <t>bool</t>
   </si>
   <si>
-    <t>category</t>
-  </si>
-  <si>
-    <t>Booleana (0/1)</t>
-  </si>
-  <si>
-    <t>int64</t>
+    <t>str</t>
+  </si>
+  <si>
+    <t>boolean</t>
   </si>
   <si>
     <t>71.46%</t>
@@ -358,54 +352,39 @@
     <t>44.71%</t>
   </si>
   <si>
+    <t>67.61%</t>
+  </si>
+  <si>
+    <t>62.50%</t>
+  </si>
+  <si>
+    <t>54.51%</t>
+  </si>
+  <si>
+    <t>48.21%</t>
+  </si>
+  <si>
+    <t>42.10%</t>
+  </si>
+  <si>
+    <t>54.11%</t>
+  </si>
+  <si>
+    <t>47.44%</t>
+  </si>
+  <si>
+    <t>96.81%</t>
+  </si>
+  <si>
+    <t>29.81%</t>
+  </si>
+  <si>
+    <t>42.50%</t>
+  </si>
+  <si>
     <t>0.00%</t>
   </si>
   <si>
-    <t>67.61%</t>
-  </si>
-  <si>
-    <t>62.50%</t>
-  </si>
-  <si>
-    <t>42.23%</t>
-  </si>
-  <si>
-    <t>35.93%</t>
-  </si>
-  <si>
-    <t>29.81%</t>
-  </si>
-  <si>
-    <t>55.33%</t>
-  </si>
-  <si>
-    <t>50.21%</t>
-  </si>
-  <si>
-    <t>41.83%</t>
-  </si>
-  <si>
-    <t>35.16%</t>
-  </si>
-  <si>
-    <t>96.81%</t>
-  </si>
-  <si>
-    <t>44.93%</t>
-  </si>
-  <si>
-    <t>38.09%</t>
-  </si>
-  <si>
-    <t>54.51%</t>
-  </si>
-  <si>
-    <t>48.21%</t>
-  </si>
-  <si>
-    <t>42.50%</t>
-  </si>
-  <si>
     <t>0.96%</t>
   </si>
   <si>
@@ -418,6 +397,9 @@
     <t>7.49%</t>
   </si>
   <si>
+    <t>33.00%</t>
+  </si>
+  <si>
     <t>7.76%</t>
   </si>
   <si>
@@ -478,19 +460,13 @@
     <t>0.01%</t>
   </si>
   <si>
-    <t>38.91%</t>
+    <t>0.40%</t>
   </si>
   <si>
     <t>12.29%</t>
   </si>
   <si>
-    <t>12.69%</t>
-  </si>
-  <si>
-    <t>14.90%</t>
-  </si>
-  <si>
-    <t>67.00%</t>
+    <t>2.61%</t>
   </si>
   <si>
     <t>71.14%</t>
@@ -505,7 +481,7 @@
     <t>68.07%</t>
   </si>
   <si>
-    <t>90.90%</t>
+    <t>57.90%</t>
   </si>
   <si>
     <t>9.26%</t>
@@ -544,6 +520,18 @@
     <t>0.90%</t>
   </si>
   <si>
+    <t>'s-Hertogenbosch</t>
+  </si>
+  <si>
+    <t>$NOT</t>
+  </si>
+  <si>
+    <t>Żelazowa Wola</t>
+  </si>
+  <si>
+    <t>酷狗文化</t>
+  </si>
+  <si>
     <t>1450.44</t>
   </si>
   <si>
@@ -565,34 +553,34 @@
     <t>7062.28</t>
   </si>
   <si>
-    <t>9.01</t>
-  </si>
-  <si>
-    <t>13.15</t>
-  </si>
-  <si>
-    <t>18.09</t>
-  </si>
-  <si>
-    <t>2.06</t>
-  </si>
-  <si>
-    <t>2.86</t>
-  </si>
-  <si>
-    <t>3.52</t>
-  </si>
-  <si>
-    <t>1.16</t>
-  </si>
-  <si>
-    <t>1.34</t>
-  </si>
-  <si>
-    <t>11.01</t>
-  </si>
-  <si>
-    <t>16.42</t>
+    <t>11.44</t>
+  </si>
+  <si>
+    <t>16.27</t>
+  </si>
+  <si>
+    <t>21.93</t>
+  </si>
+  <si>
+    <t>2.61</t>
+  </si>
+  <si>
+    <t>3.54</t>
+  </si>
+  <si>
+    <t>4.26</t>
+  </si>
+  <si>
+    <t>1.60</t>
+  </si>
+  <si>
+    <t>1.78</t>
+  </si>
+  <si>
+    <t>13.96</t>
+  </si>
+  <si>
+    <t>20.26</t>
   </si>
   <si>
     <t>8.70</t>
@@ -601,13 +589,13 @@
     <t>24.30</t>
   </si>
   <si>
-    <t>9.89</t>
-  </si>
-  <si>
-    <t>14.23</t>
-  </si>
-  <si>
-    <t>20.32</t>
+    <t>12.73</t>
+  </si>
+  <si>
+    <t>17.75</t>
+  </si>
+  <si>
+    <t>24.63</t>
   </si>
   <si>
     <t>6.94</t>
@@ -742,12 +730,6 @@
     <t>12576535.32</t>
   </si>
   <si>
-    <t>4276 (61.09%)</t>
-  </si>
-  <si>
-    <t>223 (3.19%)</t>
-  </si>
-  <si>
     <t>2020 (28.86%)</t>
   </si>
   <si>
@@ -757,22 +739,13 @@
     <t>637 (9.10%)</t>
   </si>
   <si>
-    <t>2724 (38.91%)</t>
-  </si>
-  <si>
-    <t>4690 (67.00%)</t>
-  </si>
-  <si>
-    <t>6777 (96.81%)</t>
-  </si>
-  <si>
     <t>4980 (71.14%)</t>
   </si>
   <si>
     <t>4765 (68.07%)</t>
   </si>
   <si>
-    <t>6363 (90.90%)</t>
+    <t>4053 (57.90%)</t>
   </si>
 </sst>
 </file>
@@ -1134,7 +1107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="13" width="20.7109375" customWidth="1"/>
@@ -1189,19 +1162,19 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D2">
         <v>5002</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H2">
         <v>9</v>
@@ -1210,16 +1183,16 @@
         <v>66275</v>
       </c>
       <c r="J2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="K2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1230,19 +1203,19 @@
         <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D3">
         <v>4579</v>
       </c>
       <c r="E3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H3">
         <v>20</v>
@@ -1251,16 +1224,16 @@
         <v>50153</v>
       </c>
       <c r="J3" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K3" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L3" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M3" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1271,19 +1244,19 @@
         <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D4">
         <v>5002</v>
       </c>
       <c r="E4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -1292,16 +1265,16 @@
         <v>1498</v>
       </c>
       <c r="J4" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="K4" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L4" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M4" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1312,19 +1285,19 @@
         <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D5">
         <v>4579</v>
       </c>
       <c r="E5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1333,16 +1306,16 @@
         <v>22055</v>
       </c>
       <c r="J5" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="K5" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L5" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M5" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1353,19 +1326,19 @@
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D6">
         <v>4005</v>
       </c>
       <c r="E6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H6">
         <v>60</v>
@@ -1374,16 +1347,16 @@
         <v>90000</v>
       </c>
       <c r="J6" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="K6" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L6" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M6" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1394,19 +1367,19 @@
         <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D7">
         <v>3526</v>
       </c>
       <c r="E7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1415,16 +1388,16 @@
         <v>250000</v>
       </c>
       <c r="J7" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="K7" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L7" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M7" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1435,19 +1408,19 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D8">
         <v>3130</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H8">
         <v>75</v>
@@ -1456,16 +1429,16 @@
         <v>130975</v>
       </c>
       <c r="J8" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K8" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L8" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M8" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1476,37 +1449,37 @@
         <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>4733</v>
       </c>
       <c r="E9" t="s">
-        <v>114</v>
-      </c>
-      <c r="F9">
-        <v>2724</v>
+        <v>112</v>
+      </c>
+      <c r="F9" t="s">
+        <v>146</v>
       </c>
       <c r="G9" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="H9" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I9" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J9" t="s">
-        <v>152</v>
-      </c>
-      <c r="K9" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="K9">
+        <v>14</v>
       </c>
       <c r="L9" t="s">
-        <v>242</v>
+        <v>146</v>
       </c>
       <c r="M9" t="s">
-        <v>247</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1517,37 +1490,37 @@
         <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D10">
-        <v>4733</v>
+        <v>4375</v>
       </c>
       <c r="E10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F10" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="G10" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="H10" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I10" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J10" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="K10">
         <v>14</v>
       </c>
       <c r="L10" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M10" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1558,37 +1531,37 @@
         <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D11">
-        <v>4375</v>
+        <v>3816</v>
       </c>
       <c r="E11" t="s">
-        <v>116</v>
-      </c>
-      <c r="F11" t="s">
-        <v>152</v>
+        <v>114</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>152</v>
-      </c>
-      <c r="H11" t="s">
-        <v>152</v>
-      </c>
-      <c r="I11" t="s">
-        <v>152</v>
+        <v>122</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>84</v>
       </c>
       <c r="J11" t="s">
-        <v>152</v>
-      </c>
-      <c r="K11">
-        <v>14</v>
+        <v>179</v>
+      </c>
+      <c r="K11" t="s">
+        <v>146</v>
       </c>
       <c r="L11" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M11" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -1599,37 +1572,37 @@
         <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D12">
-        <v>2956</v>
+        <v>3375</v>
       </c>
       <c r="E12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F12">
-        <v>860</v>
+        <v>0</v>
       </c>
       <c r="G12" t="s">
-        <v>155</v>
+        <v>122</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="J12" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="K12" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L12" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M12" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1640,37 +1613,37 @@
         <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D13">
-        <v>2515</v>
+        <v>2947</v>
       </c>
       <c r="E13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F13">
-        <v>860</v>
+        <v>28</v>
       </c>
       <c r="G13" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="I13">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="J13" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="K13" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L13" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M13" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1681,37 +1654,37 @@
         <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D14">
-        <v>2087</v>
+        <v>3816</v>
       </c>
       <c r="E14" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="F14">
-        <v>888</v>
+        <v>0</v>
       </c>
       <c r="G14" t="s">
-        <v>156</v>
+        <v>122</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14">
-        <v>140</v>
+        <v>26</v>
       </c>
       <c r="J14" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="K14" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L14" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M14" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -1722,37 +1695,37 @@
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D15">
-        <v>2956</v>
+        <v>3375</v>
       </c>
       <c r="E15" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F15">
-        <v>860</v>
+        <v>0</v>
       </c>
       <c r="G15" t="s">
-        <v>155</v>
+        <v>122</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J15" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="K15" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L15" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M15" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -1763,37 +1736,37 @@
         <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D16">
-        <v>2515</v>
+        <v>2947</v>
       </c>
       <c r="E16" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F16">
-        <v>860</v>
+        <v>28</v>
       </c>
       <c r="G16" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="H16">
         <v>0</v>
       </c>
       <c r="I16">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="J16" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="K16" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L16" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M16" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1804,37 +1777,37 @@
         <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D17">
-        <v>2087</v>
+        <v>4733</v>
       </c>
       <c r="E17" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="F17">
-        <v>888</v>
+        <v>0</v>
       </c>
       <c r="G17" t="s">
-        <v>156</v>
+        <v>122</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="J17" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="K17" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L17" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M17" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1845,37 +1818,37 @@
         <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D18">
-        <v>3873</v>
+        <v>4375</v>
       </c>
       <c r="E18" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="F18">
-        <v>860</v>
+        <v>0</v>
       </c>
       <c r="G18" t="s">
-        <v>155</v>
+        <v>122</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J18" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="K18" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L18" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M18" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -1886,37 +1859,37 @@
         <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D19">
-        <v>3515</v>
+        <v>3788</v>
       </c>
       <c r="E19" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F19">
-        <v>860</v>
+        <v>0</v>
       </c>
       <c r="G19" t="s">
-        <v>155</v>
+        <v>122</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="J19" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="K19" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L19" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M19" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1927,37 +1900,37 @@
         <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D20">
-        <v>2928</v>
+        <v>3321</v>
       </c>
       <c r="E20" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F20">
-        <v>860</v>
+        <v>0</v>
       </c>
       <c r="G20" t="s">
-        <v>155</v>
+        <v>122</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20">
-        <v>90</v>
+        <v>129</v>
       </c>
       <c r="J20" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="K20" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L20" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M20" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -1968,37 +1941,37 @@
         <v>38</v>
       </c>
       <c r="C21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D21">
-        <v>2461</v>
+        <v>6777</v>
       </c>
       <c r="E21" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F21">
-        <v>860</v>
+        <v>0</v>
       </c>
       <c r="G21" t="s">
-        <v>155</v>
+        <v>122</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="J21" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="K21" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L21" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M21" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -2009,37 +1982,37 @@
         <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D22">
-        <v>6777</v>
+        <v>2087</v>
       </c>
       <c r="E22" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>860</v>
       </c>
       <c r="G22" t="s">
-        <v>114</v>
+        <v>149</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22">
-        <v>118</v>
+        <v>179</v>
       </c>
       <c r="J22" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="K22" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L22" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M22" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -2050,37 +2023,37 @@
         <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D23">
-        <v>2087</v>
+        <v>4005</v>
       </c>
       <c r="E23" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="F23">
-        <v>860</v>
+        <v>0</v>
       </c>
       <c r="G23" t="s">
-        <v>155</v>
+        <v>122</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23">
-        <v>179</v>
+        <v>86</v>
       </c>
       <c r="J23" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="K23" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L23" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M23" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -2091,37 +2064,37 @@
         <v>41</v>
       </c>
       <c r="C24" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D24">
-        <v>3145</v>
+        <v>3526</v>
       </c>
       <c r="E24" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="F24">
-        <v>860</v>
+        <v>0</v>
       </c>
       <c r="G24" t="s">
-        <v>155</v>
+        <v>122</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="J24" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K24" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L24" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M24" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -2132,37 +2105,37 @@
         <v>42</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D25">
-        <v>2666</v>
+        <v>2947</v>
       </c>
       <c r="E25" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="F25">
-        <v>860</v>
+        <v>183</v>
       </c>
       <c r="G25" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="H25">
         <v>0</v>
       </c>
       <c r="I25">
-        <v>112</v>
+        <v>160</v>
       </c>
       <c r="J25" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="K25" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L25" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M25" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -2173,37 +2146,37 @@
         <v>43</v>
       </c>
       <c r="C26" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D26">
-        <v>2087</v>
+        <v>3816</v>
       </c>
       <c r="E26" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="F26">
-        <v>1043</v>
+        <v>0</v>
       </c>
       <c r="G26" t="s">
-        <v>157</v>
+        <v>122</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26">
-        <v>160</v>
+        <v>72</v>
       </c>
       <c r="J26" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="K26" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L26" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M26" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -2214,37 +2187,37 @@
         <v>44</v>
       </c>
       <c r="C27" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D27">
-        <v>2087</v>
+        <v>3375</v>
       </c>
       <c r="E27" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F27">
-        <v>4690</v>
+        <v>0</v>
       </c>
       <c r="G27" t="s">
-        <v>158</v>
-      </c>
-      <c r="H27" t="s">
-        <v>152</v>
-      </c>
-      <c r="I27" t="s">
-        <v>152</v>
+        <v>122</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27">
+        <v>129</v>
       </c>
       <c r="J27" t="s">
-        <v>152</v>
+        <v>195</v>
       </c>
       <c r="K27" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L27" t="s">
-        <v>243</v>
+        <v>146</v>
       </c>
       <c r="M27" t="s">
-        <v>248</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -2255,37 +2228,37 @@
         <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>2975</v>
       </c>
       <c r="E28" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="F28">
-        <v>6777</v>
+        <v>0</v>
       </c>
       <c r="G28" t="s">
-        <v>124</v>
-      </c>
-      <c r="H28" t="s">
-        <v>152</v>
-      </c>
-      <c r="I28" t="s">
-        <v>152</v>
+        <v>122</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
+      <c r="I28">
+        <v>170</v>
       </c>
       <c r="J28" t="s">
-        <v>152</v>
+        <v>196</v>
       </c>
       <c r="K28" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L28" t="s">
-        <v>243</v>
+        <v>146</v>
       </c>
       <c r="M28" t="s">
-        <v>249</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -2296,37 +2269,37 @@
         <v>46</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D29">
-        <v>3816</v>
+        <v>4005</v>
       </c>
       <c r="E29" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
       <c r="G29" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H29">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="I29">
-        <v>72</v>
+        <v>3185238</v>
       </c>
       <c r="J29" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K29" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L29" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M29" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -2337,37 +2310,37 @@
         <v>47</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D30">
-        <v>3375</v>
+        <v>3526</v>
       </c>
       <c r="E30" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="s">
-        <v>114</v>
+        <v>147</v>
       </c>
       <c r="H30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I30">
-        <v>129</v>
+        <v>3350782</v>
       </c>
       <c r="J30" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K30" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L30" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M30" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -2378,42 +2351,42 @@
         <v>48</v>
       </c>
       <c r="C31" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D31">
-        <v>2975</v>
+        <v>3130</v>
       </c>
       <c r="E31" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H31">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="I31">
-        <v>170</v>
+        <v>4167910</v>
       </c>
       <c r="J31" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K31" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L31" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M31" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:13">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B32" t="s">
         <v>49</v>
@@ -2422,116 +2395,116 @@
         <v>104</v>
       </c>
       <c r="D32">
-        <v>4005</v>
+        <v>0</v>
       </c>
       <c r="E32" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="F32">
-        <v>0</v>
+        <v>4980</v>
       </c>
       <c r="G32" t="s">
-        <v>114</v>
-      </c>
-      <c r="H32">
-        <v>60</v>
-      </c>
-      <c r="I32">
-        <v>3185238</v>
+        <v>151</v>
+      </c>
+      <c r="H32" t="s">
+        <v>146</v>
+      </c>
+      <c r="I32" t="s">
+        <v>146</v>
       </c>
       <c r="J32" t="s">
-        <v>201</v>
+        <v>146</v>
       </c>
       <c r="K32" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L32" t="s">
-        <v>152</v>
+        <v>238</v>
       </c>
       <c r="M32" t="s">
-        <v>152</v>
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:13">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B33" t="s">
         <v>50</v>
       </c>
       <c r="C33" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D33">
-        <v>3526</v>
+        <v>0</v>
       </c>
       <c r="E33" t="s">
-        <v>112</v>
-      </c>
-      <c r="F33">
-        <v>1</v>
+        <v>122</v>
+      </c>
+      <c r="F33" t="s">
+        <v>146</v>
       </c>
       <c r="G33" t="s">
-        <v>153</v>
-      </c>
-      <c r="H33">
-        <v>0</v>
-      </c>
-      <c r="I33">
-        <v>3350782</v>
+        <v>146</v>
+      </c>
+      <c r="H33" t="s">
+        <v>146</v>
+      </c>
+      <c r="I33" t="s">
+        <v>146</v>
       </c>
       <c r="J33" t="s">
-        <v>202</v>
-      </c>
-      <c r="K33" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="K33">
+        <v>5</v>
       </c>
       <c r="L33" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M33" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="34" spans="1:13">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B34" t="s">
         <v>51</v>
       </c>
       <c r="C34" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D34">
-        <v>3130</v>
+        <v>0</v>
       </c>
       <c r="E34" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>372</v>
       </c>
       <c r="G34" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="H34">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="I34">
-        <v>4167910</v>
+        <v>100</v>
       </c>
       <c r="J34" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="K34" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L34" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M34" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -2542,37 +2515,37 @@
         <v>52</v>
       </c>
       <c r="C35" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D35">
         <v>0</v>
       </c>
       <c r="E35" t="s">
-        <v>114</v>
-      </c>
-      <c r="F35">
-        <v>4980</v>
+        <v>122</v>
+      </c>
+      <c r="F35" t="s">
+        <v>146</v>
       </c>
       <c r="G35" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="H35" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I35" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J35" t="s">
-        <v>152</v>
-      </c>
-      <c r="K35" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="K35">
+        <v>5</v>
       </c>
       <c r="L35" t="s">
-        <v>244</v>
+        <v>146</v>
       </c>
       <c r="M35" t="s">
-        <v>250</v>
+        <v>146</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -2583,37 +2556,37 @@
         <v>53</v>
       </c>
       <c r="C36" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D36">
         <v>0</v>
       </c>
       <c r="E36" t="s">
-        <v>114</v>
-      </c>
-      <c r="F36" t="s">
-        <v>152</v>
+        <v>122</v>
+      </c>
+      <c r="F36">
+        <v>82</v>
       </c>
       <c r="G36" t="s">
-        <v>152</v>
-      </c>
-      <c r="H36" t="s">
-        <v>152</v>
-      </c>
-      <c r="I36" t="s">
-        <v>152</v>
+        <v>153</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>100</v>
       </c>
       <c r="J36" t="s">
-        <v>152</v>
-      </c>
-      <c r="K36">
-        <v>5</v>
+        <v>201</v>
+      </c>
+      <c r="K36" t="s">
+        <v>146</v>
       </c>
       <c r="L36" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M36" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -2624,37 +2597,37 @@
         <v>54</v>
       </c>
       <c r="C37" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D37">
         <v>0</v>
       </c>
       <c r="E37" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="F37">
-        <v>372</v>
+        <v>0</v>
       </c>
       <c r="G37" t="s">
-        <v>160</v>
+        <v>122</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I37">
-        <v>100</v>
+        <v>14847778</v>
       </c>
       <c r="J37" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="K37" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L37" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M37" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -2665,37 +2638,37 @@
         <v>55</v>
       </c>
       <c r="C38" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D38">
         <v>0</v>
       </c>
       <c r="E38" t="s">
-        <v>114</v>
-      </c>
-      <c r="F38" t="s">
-        <v>152</v>
+        <v>122</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
       </c>
       <c r="G38" t="s">
-        <v>152</v>
-      </c>
-      <c r="H38" t="s">
-        <v>152</v>
-      </c>
-      <c r="I38" t="s">
-        <v>152</v>
+        <v>122</v>
+      </c>
+      <c r="H38">
+        <v>1</v>
+      </c>
+      <c r="I38">
+        <v>458903</v>
       </c>
       <c r="J38" t="s">
-        <v>152</v>
-      </c>
-      <c r="K38">
-        <v>5</v>
+        <v>203</v>
+      </c>
+      <c r="K38" t="s">
+        <v>146</v>
       </c>
       <c r="L38" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M38" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -2706,37 +2679,37 @@
         <v>56</v>
       </c>
       <c r="C39" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="D39">
         <v>0</v>
       </c>
       <c r="E39" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="F39">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="G39" t="s">
-        <v>161</v>
+        <v>122</v>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>26.02413665904167</v>
       </c>
       <c r="I39">
-        <v>100</v>
+        <v>99.38711679376492</v>
       </c>
       <c r="J39" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K39" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L39" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M39" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" spans="1:13">
@@ -2747,37 +2720,37 @@
         <v>57</v>
       </c>
       <c r="C40" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D40">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="E40" t="s">
-        <v>114</v>
-      </c>
-      <c r="F40">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="F40" t="s">
+        <v>146</v>
       </c>
       <c r="G40" t="s">
-        <v>114</v>
-      </c>
-      <c r="H40">
-        <v>2</v>
-      </c>
-      <c r="I40">
-        <v>14847778</v>
+        <v>146</v>
+      </c>
+      <c r="H40" t="s">
+        <v>146</v>
+      </c>
+      <c r="I40" t="s">
+        <v>146</v>
       </c>
       <c r="J40" t="s">
-        <v>206</v>
-      </c>
-      <c r="K40" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="K40">
+        <v>112</v>
       </c>
       <c r="L40" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M40" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -2788,37 +2761,37 @@
         <v>58</v>
       </c>
       <c r="C41" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D41">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="E41" t="s">
-        <v>114</v>
-      </c>
-      <c r="F41">
-        <v>0</v>
+        <v>123</v>
+      </c>
+      <c r="F41" t="s">
+        <v>146</v>
       </c>
       <c r="G41" t="s">
-        <v>114</v>
-      </c>
-      <c r="H41">
-        <v>1</v>
-      </c>
-      <c r="I41">
-        <v>458903</v>
+        <v>146</v>
+      </c>
+      <c r="H41" t="s">
+        <v>146</v>
+      </c>
+      <c r="I41" t="s">
+        <v>146</v>
       </c>
       <c r="J41" t="s">
-        <v>207</v>
-      </c>
-      <c r="K41" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="K41">
+        <v>6</v>
       </c>
       <c r="L41" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M41" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -2829,37 +2802,37 @@
         <v>59</v>
       </c>
       <c r="C42" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D42">
-        <v>0</v>
+        <v>4561</v>
       </c>
       <c r="E42" t="s">
-        <v>114</v>
-      </c>
-      <c r="F42">
-        <v>0</v>
+        <v>124</v>
+      </c>
+      <c r="F42" t="s">
+        <v>146</v>
       </c>
       <c r="G42" t="s">
-        <v>114</v>
-      </c>
-      <c r="H42">
-        <v>26.02413665904167</v>
-      </c>
-      <c r="I42">
-        <v>99.38711679376492</v>
+        <v>146</v>
+      </c>
+      <c r="H42" t="s">
+        <v>146</v>
+      </c>
+      <c r="I42" t="s">
+        <v>146</v>
       </c>
       <c r="J42" t="s">
-        <v>208</v>
-      </c>
-      <c r="K42" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="K42">
+        <v>11</v>
       </c>
       <c r="L42" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M42" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -2870,37 +2843,37 @@
         <v>60</v>
       </c>
       <c r="C43" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D43">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="E43" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="F43" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="G43" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="H43" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I43" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J43" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="K43">
-        <v>112</v>
+        <v>12</v>
       </c>
       <c r="L43" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M43" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -2911,37 +2884,37 @@
         <v>61</v>
       </c>
       <c r="C44" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D44">
-        <v>67</v>
+        <v>2608</v>
       </c>
       <c r="E44" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F44" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="G44" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="H44" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="I44" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="J44" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="K44">
-        <v>7</v>
+        <v>1083</v>
       </c>
       <c r="L44" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M44" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -2955,34 +2928,34 @@
         <v>106</v>
       </c>
       <c r="D45">
-        <v>4561</v>
+        <v>524</v>
       </c>
       <c r="E45" t="s">
-        <v>131</v>
-      </c>
-      <c r="F45" t="s">
-        <v>152</v>
+        <v>126</v>
+      </c>
+      <c r="F45">
+        <v>4765</v>
       </c>
       <c r="G45" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H45" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I45" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J45" t="s">
-        <v>152</v>
-      </c>
-      <c r="K45">
-        <v>11</v>
+        <v>146</v>
+      </c>
+      <c r="K45" t="s">
+        <v>146</v>
       </c>
       <c r="L45" t="s">
-        <v>152</v>
+        <v>239</v>
       </c>
       <c r="M45" t="s">
-        <v>152</v>
+        <v>242</v>
       </c>
     </row>
     <row r="46" spans="1:13">
@@ -2996,34 +2969,34 @@
         <v>106</v>
       </c>
       <c r="D46">
-        <v>0</v>
+        <v>2310</v>
       </c>
       <c r="E46" t="s">
-        <v>114</v>
-      </c>
-      <c r="F46" t="s">
-        <v>152</v>
+        <v>127</v>
+      </c>
+      <c r="F46">
+        <v>4053</v>
       </c>
       <c r="G46" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H46" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I46" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J46" t="s">
-        <v>152</v>
-      </c>
-      <c r="K46">
-        <v>12</v>
+        <v>146</v>
+      </c>
+      <c r="K46" t="s">
+        <v>146</v>
       </c>
       <c r="L46" t="s">
-        <v>152</v>
+        <v>240</v>
       </c>
       <c r="M46" t="s">
-        <v>152</v>
+        <v>243</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -3034,37 +3007,37 @@
         <v>64</v>
       </c>
       <c r="C47" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D47">
-        <v>2608</v>
+        <v>0</v>
       </c>
       <c r="E47" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="F47" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="G47" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="H47" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I47" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J47" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="K47">
-        <v>1083</v>
+        <v>339</v>
       </c>
       <c r="L47" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M47" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -3075,37 +3048,37 @@
         <v>65</v>
       </c>
       <c r="C48" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D48">
-        <v>524</v>
+        <v>0</v>
       </c>
       <c r="E48" t="s">
-        <v>133</v>
-      </c>
-      <c r="F48">
-        <v>4765</v>
+        <v>122</v>
+      </c>
+      <c r="F48" t="s">
+        <v>146</v>
       </c>
       <c r="G48" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="H48" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I48" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J48" t="s">
-        <v>152</v>
-      </c>
-      <c r="K48" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="K48">
+        <v>4</v>
       </c>
       <c r="L48" t="s">
-        <v>245</v>
+        <v>146</v>
       </c>
       <c r="M48" t="s">
-        <v>251</v>
+        <v>146</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -3116,37 +3089,37 @@
         <v>66</v>
       </c>
       <c r="C49" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D49">
         <v>0</v>
       </c>
       <c r="E49" t="s">
-        <v>114</v>
-      </c>
-      <c r="F49">
-        <v>6363</v>
+        <v>122</v>
+      </c>
+      <c r="F49" t="s">
+        <v>146</v>
       </c>
       <c r="G49" t="s">
-        <v>163</v>
+        <v>146</v>
       </c>
       <c r="H49" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I49" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J49" t="s">
-        <v>152</v>
-      </c>
-      <c r="K49" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="K49">
+        <v>11</v>
       </c>
       <c r="L49" t="s">
-        <v>246</v>
+        <v>146</v>
       </c>
       <c r="M49" t="s">
-        <v>252</v>
+        <v>146</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -3157,160 +3130,160 @@
         <v>67</v>
       </c>
       <c r="C50" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D50">
-        <v>0</v>
+        <v>524</v>
       </c>
       <c r="E50" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="F50" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="G50" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="H50" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="I50" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="J50" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="K50">
-        <v>339</v>
+        <v>3574</v>
       </c>
       <c r="L50" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M50" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="51" spans="1:13">
       <c r="A51" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B51" t="s">
         <v>68</v>
       </c>
       <c r="C51" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D51">
-        <v>0</v>
+        <v>543</v>
       </c>
       <c r="E51" t="s">
-        <v>114</v>
-      </c>
-      <c r="F51" t="s">
-        <v>152</v>
+        <v>128</v>
+      </c>
+      <c r="F51">
+        <v>648</v>
       </c>
       <c r="G51" t="s">
-        <v>152</v>
-      </c>
-      <c r="H51" t="s">
-        <v>152</v>
-      </c>
-      <c r="I51" t="s">
-        <v>152</v>
+        <v>156</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51">
+        <v>43152895</v>
       </c>
       <c r="J51" t="s">
-        <v>152</v>
-      </c>
-      <c r="K51">
-        <v>4</v>
+        <v>205</v>
+      </c>
+      <c r="K51" t="s">
+        <v>146</v>
       </c>
       <c r="L51" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M51" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="52" spans="1:13">
       <c r="A52" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B52" t="s">
         <v>69</v>
       </c>
       <c r="C52" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D52">
-        <v>0</v>
+        <v>543</v>
       </c>
       <c r="E52" t="s">
-        <v>114</v>
-      </c>
-      <c r="F52" t="s">
-        <v>152</v>
+        <v>128</v>
+      </c>
+      <c r="F52">
+        <v>4</v>
       </c>
       <c r="G52" t="s">
-        <v>152</v>
-      </c>
-      <c r="H52" t="s">
-        <v>152</v>
-      </c>
-      <c r="I52" t="s">
-        <v>152</v>
+        <v>157</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52">
+        <v>75271226</v>
       </c>
       <c r="J52" t="s">
-        <v>152</v>
-      </c>
-      <c r="K52">
-        <v>11</v>
+        <v>206</v>
+      </c>
+      <c r="K52" t="s">
+        <v>146</v>
       </c>
       <c r="L52" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M52" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="53" spans="1:13">
       <c r="A53" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B53" t="s">
         <v>70</v>
       </c>
       <c r="C53" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D53">
-        <v>524</v>
+        <v>226</v>
       </c>
       <c r="E53" t="s">
-        <v>133</v>
-      </c>
-      <c r="F53" t="s">
-        <v>152</v>
+        <v>129</v>
+      </c>
+      <c r="F53">
+        <v>110</v>
       </c>
       <c r="G53" t="s">
-        <v>152</v>
-      </c>
-      <c r="H53" t="s">
-        <v>152</v>
-      </c>
-      <c r="I53" t="s">
-        <v>152</v>
+        <v>158</v>
+      </c>
+      <c r="H53">
+        <v>0</v>
+      </c>
+      <c r="I53">
+        <v>2473</v>
       </c>
       <c r="J53" t="s">
-        <v>152</v>
-      </c>
-      <c r="K53">
-        <v>3574</v>
+        <v>207</v>
+      </c>
+      <c r="K53" t="s">
+        <v>146</v>
       </c>
       <c r="L53" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M53" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -3321,37 +3294,37 @@
         <v>71</v>
       </c>
       <c r="C54" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D54">
-        <v>543</v>
+        <v>226</v>
       </c>
       <c r="E54" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F54">
-        <v>648</v>
+        <v>0</v>
       </c>
       <c r="G54" t="s">
-        <v>164</v>
+        <v>122</v>
       </c>
       <c r="H54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I54">
-        <v>43152895</v>
+        <v>6407</v>
       </c>
       <c r="J54" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K54" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L54" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M54" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -3362,37 +3335,37 @@
         <v>72</v>
       </c>
       <c r="C55" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D55">
-        <v>543</v>
+        <v>799</v>
       </c>
       <c r="E55" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F55">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="G55" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="H55">
         <v>0</v>
       </c>
       <c r="I55">
-        <v>75271226</v>
+        <v>1570</v>
       </c>
       <c r="J55" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K55" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L55" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M55" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -3403,37 +3376,37 @@
         <v>73</v>
       </c>
       <c r="C56" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D56">
-        <v>226</v>
+        <v>799</v>
       </c>
       <c r="E56" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F56">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="G56" t="s">
-        <v>166</v>
+        <v>122</v>
       </c>
       <c r="H56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I56">
-        <v>2473</v>
+        <v>1680</v>
       </c>
       <c r="J56" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K56" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L56" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M56" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -3444,37 +3417,37 @@
         <v>74</v>
       </c>
       <c r="C57" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D57">
-        <v>226</v>
+        <v>543</v>
       </c>
       <c r="E57" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="F57">
-        <v>0</v>
+        <v>648</v>
       </c>
       <c r="G57" t="s">
-        <v>114</v>
+        <v>156</v>
       </c>
       <c r="H57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I57">
-        <v>6407</v>
+        <v>413</v>
       </c>
       <c r="J57" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K57" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L57" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M57" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -3485,37 +3458,37 @@
         <v>75</v>
       </c>
       <c r="C58" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D58">
-        <v>799</v>
+        <v>543</v>
       </c>
       <c r="E58" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="F58">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G58" t="s">
-        <v>167</v>
+        <v>122</v>
       </c>
       <c r="H58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I58">
-        <v>1570</v>
+        <v>2024</v>
       </c>
       <c r="J58" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="K58" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L58" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M58" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -3526,37 +3499,37 @@
         <v>76</v>
       </c>
       <c r="C59" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D59">
-        <v>799</v>
+        <v>11</v>
       </c>
       <c r="E59" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="F59">
-        <v>0</v>
+        <v>218</v>
       </c>
       <c r="G59" t="s">
-        <v>114</v>
+        <v>160</v>
       </c>
       <c r="H59">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I59">
-        <v>1680</v>
+        <v>2393</v>
       </c>
       <c r="J59" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K59" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L59" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M59" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -3567,37 +3540,37 @@
         <v>77</v>
       </c>
       <c r="C60" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D60">
-        <v>543</v>
+        <v>11</v>
       </c>
       <c r="E60" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="F60">
-        <v>648</v>
+        <v>0</v>
       </c>
       <c r="G60" t="s">
-        <v>164</v>
+        <v>122</v>
       </c>
       <c r="H60">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I60">
-        <v>413</v>
+        <v>3376367</v>
       </c>
       <c r="J60" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K60" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L60" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M60" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -3608,37 +3581,37 @@
         <v>78</v>
       </c>
       <c r="C61" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D61">
-        <v>543</v>
+        <v>431</v>
       </c>
       <c r="E61" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F61">
-        <v>0</v>
+        <v>703</v>
       </c>
       <c r="G61" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="H61">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I61">
-        <v>2024</v>
+        <v>204</v>
       </c>
       <c r="J61" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K61" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L61" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M61" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -3649,37 +3622,37 @@
         <v>79</v>
       </c>
       <c r="C62" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D62">
-        <v>11</v>
+        <v>431</v>
       </c>
       <c r="E62" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F62">
-        <v>218</v>
+        <v>0</v>
       </c>
       <c r="G62" t="s">
-        <v>168</v>
+        <v>122</v>
       </c>
       <c r="H62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I62">
-        <v>2393</v>
+        <v>1271</v>
       </c>
       <c r="J62" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="K62" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L62" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M62" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="63" spans="1:13">
@@ -3690,37 +3663,37 @@
         <v>80</v>
       </c>
       <c r="C63" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D63">
         <v>11</v>
       </c>
       <c r="E63" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F63">
-        <v>0</v>
+        <v>244</v>
       </c>
       <c r="G63" t="s">
-        <v>114</v>
+        <v>162</v>
       </c>
       <c r="H63">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I63">
-        <v>3376367</v>
+        <v>401578965</v>
       </c>
       <c r="J63" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K63" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L63" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M63" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -3731,160 +3704,160 @@
         <v>81</v>
       </c>
       <c r="C64" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D64">
-        <v>431</v>
+        <v>549</v>
       </c>
       <c r="E64" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F64">
-        <v>703</v>
+        <v>0</v>
       </c>
       <c r="G64" t="s">
-        <v>169</v>
+        <v>122</v>
       </c>
       <c r="H64">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I64">
-        <v>204</v>
+        <v>14446891354</v>
       </c>
       <c r="J64" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K64" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L64" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M64" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="65" spans="1:13">
       <c r="A65" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B65" t="s">
         <v>82</v>
       </c>
       <c r="C65" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D65">
-        <v>431</v>
+        <v>606</v>
       </c>
       <c r="E65" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F65">
         <v>0</v>
       </c>
       <c r="G65" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H65">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I65">
-        <v>1271</v>
+        <v>415101450</v>
       </c>
       <c r="J65" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="K65" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L65" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M65" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="66" spans="1:13">
       <c r="A66" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B66" t="s">
         <v>83</v>
       </c>
       <c r="C66" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D66">
-        <v>11</v>
+        <v>2199</v>
       </c>
       <c r="E66" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F66">
-        <v>244</v>
+        <v>0</v>
       </c>
       <c r="G66" t="s">
-        <v>170</v>
+        <v>122</v>
       </c>
       <c r="H66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I66">
-        <v>401578965</v>
+        <v>92600000</v>
       </c>
       <c r="J66" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="K66" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L66" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M66" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="67" spans="1:13">
       <c r="A67" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B67" t="s">
         <v>84</v>
       </c>
       <c r="C67" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D67">
-        <v>549</v>
+        <v>2199</v>
       </c>
       <c r="E67" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F67">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="G67" t="s">
-        <v>114</v>
+        <v>163</v>
       </c>
       <c r="H67">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I67">
-        <v>14446891354</v>
+        <v>5300000000</v>
       </c>
       <c r="J67" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K67" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L67" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M67" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -3895,37 +3868,37 @@
         <v>85</v>
       </c>
       <c r="C68" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D68">
-        <v>606</v>
+        <v>66</v>
       </c>
       <c r="E68" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F68">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G68" t="s">
-        <v>114</v>
+        <v>164</v>
       </c>
       <c r="H68">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I68">
-        <v>415101450</v>
+        <v>294275870</v>
       </c>
       <c r="J68" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="K68" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L68" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M68" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="69" spans="1:13">
@@ -3936,37 +3909,37 @@
         <v>86</v>
       </c>
       <c r="C69" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D69">
-        <v>2199</v>
+        <v>66</v>
       </c>
       <c r="E69" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F69">
         <v>0</v>
       </c>
       <c r="G69" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H69">
-        <v>1</v>
+        <v>109</v>
       </c>
       <c r="I69">
-        <v>92600000</v>
+        <v>225624671689</v>
       </c>
       <c r="J69" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K69" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L69" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M69" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="70" spans="1:13">
@@ -3977,37 +3950,37 @@
         <v>87</v>
       </c>
       <c r="C70" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D70">
-        <v>2199</v>
+        <v>67</v>
       </c>
       <c r="E70" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="F70">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="G70" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H70">
         <v>0</v>
       </c>
       <c r="I70">
-        <v>5300000000</v>
+        <v>151680251</v>
       </c>
       <c r="J70" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="K70" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L70" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M70" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="71" spans="1:13">
@@ -4018,160 +3991,160 @@
         <v>88</v>
       </c>
       <c r="C71" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D71">
-        <v>66</v>
+        <v>1773</v>
       </c>
       <c r="E71" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F71">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G71" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
       <c r="H71">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I71">
-        <v>294275870</v>
+        <v>96700769</v>
       </c>
       <c r="J71" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="K71" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L71" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M71" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="72" spans="1:13">
       <c r="A72" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B72" t="s">
         <v>89</v>
       </c>
       <c r="C72" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D72">
-        <v>66</v>
+        <v>198</v>
       </c>
       <c r="E72" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F72">
         <v>0</v>
       </c>
       <c r="G72" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H72">
-        <v>109</v>
+        <v>1</v>
       </c>
       <c r="I72">
-        <v>225624671689</v>
+        <v>20740405</v>
       </c>
       <c r="J72" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="K72" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L72" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M72" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="73" spans="1:13">
       <c r="A73" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B73" t="s">
         <v>90</v>
       </c>
       <c r="C73" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D73">
-        <v>67</v>
+        <v>670</v>
       </c>
       <c r="E73" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="F73">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G73" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
       <c r="H73">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I73">
-        <v>151680251</v>
+        <v>92298921</v>
       </c>
       <c r="J73" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="K73" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L73" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M73" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="74" spans="1:13">
       <c r="A74" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B74" t="s">
         <v>91</v>
       </c>
       <c r="C74" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D74">
-        <v>1773</v>
+        <v>470</v>
       </c>
       <c r="E74" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F74">
         <v>0</v>
       </c>
       <c r="G74" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H74">
         <v>1</v>
       </c>
       <c r="I74">
-        <v>96700769</v>
+        <v>33495855298</v>
       </c>
       <c r="J74" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="K74" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L74" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M74" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="75" spans="1:13">
@@ -4182,37 +4155,37 @@
         <v>92</v>
       </c>
       <c r="C75" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D75">
-        <v>198</v>
+        <v>17</v>
       </c>
       <c r="E75" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F75">
         <v>0</v>
       </c>
       <c r="G75" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H75">
         <v>1</v>
       </c>
       <c r="I75">
-        <v>20740405</v>
+        <v>556229266</v>
       </c>
       <c r="J75" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K75" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L75" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M75" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="76" spans="1:13">
@@ -4223,37 +4196,37 @@
         <v>93</v>
       </c>
       <c r="C76" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D76">
-        <v>670</v>
+        <v>22</v>
       </c>
       <c r="E76" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F76">
         <v>0</v>
       </c>
       <c r="G76" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H76">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I76">
-        <v>92298921</v>
+        <v>176892662</v>
       </c>
       <c r="J76" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="K76" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L76" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M76" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="77" spans="1:13">
@@ -4264,37 +4237,37 @@
         <v>94</v>
       </c>
       <c r="C77" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D77">
-        <v>470</v>
+        <v>22</v>
       </c>
       <c r="E77" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="F77">
         <v>0</v>
       </c>
       <c r="G77" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H77">
         <v>1</v>
       </c>
       <c r="I77">
-        <v>33495855298</v>
+        <v>134166866</v>
       </c>
       <c r="J77" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="K77" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L77" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M77" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -4305,37 +4278,37 @@
         <v>95</v>
       </c>
       <c r="C78" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D78">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E78" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
       <c r="F78">
         <v>0</v>
       </c>
       <c r="G78" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I78">
-        <v>556229266</v>
+        <v>1048509088</v>
       </c>
       <c r="J78" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K78" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L78" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M78" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="79" spans="1:13">
@@ -4346,160 +4319,160 @@
         <v>96</v>
       </c>
       <c r="C79" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D79">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E79" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F79">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="G79" t="s">
-        <v>114</v>
+        <v>165</v>
       </c>
       <c r="H79">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="I79">
-        <v>176892662</v>
+        <v>100</v>
       </c>
       <c r="J79" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="K79" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L79" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M79" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="80" spans="1:13">
       <c r="A80" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B80" t="s">
         <v>97</v>
       </c>
       <c r="C80" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D80">
-        <v>22</v>
+        <v>619</v>
       </c>
       <c r="E80" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F80">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="G80" t="s">
-        <v>114</v>
+        <v>166</v>
       </c>
       <c r="H80">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I80">
-        <v>134166866</v>
+        <v>200000000</v>
       </c>
       <c r="J80" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="K80" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L80" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M80" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="81" spans="1:13">
       <c r="A81" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B81" t="s">
         <v>98</v>
       </c>
       <c r="C81" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D81">
-        <v>11</v>
+        <v>619</v>
       </c>
       <c r="E81" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="F81">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="G81" t="s">
-        <v>114</v>
+        <v>167</v>
       </c>
       <c r="H81">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I81">
-        <v>1048509088</v>
+        <v>219062482434</v>
       </c>
       <c r="J81" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="K81" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L81" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M81" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="82" spans="1:13">
       <c r="A82" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B82" t="s">
         <v>99</v>
       </c>
       <c r="C82" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D82">
-        <v>8</v>
+        <v>2716</v>
       </c>
       <c r="E82" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="F82">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="G82" t="s">
-        <v>173</v>
+        <v>122</v>
       </c>
       <c r="H82">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I82">
-        <v>100</v>
+        <v>17191106</v>
       </c>
       <c r="J82" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="K82" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L82" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M82" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="83" spans="1:13">
@@ -4510,160 +4483,37 @@
         <v>100</v>
       </c>
       <c r="C83" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D83">
-        <v>619</v>
+        <v>2716</v>
       </c>
       <c r="E83" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F83">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="G83" t="s">
-        <v>174</v>
+        <v>122</v>
       </c>
       <c r="H83">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="I83">
-        <v>200000000</v>
+        <v>1456427251</v>
       </c>
       <c r="J83" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K83" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="L83" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="M83" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="84" spans="1:13">
-      <c r="A84" t="s">
-        <v>18</v>
-      </c>
-      <c r="B84" t="s">
-        <v>101</v>
-      </c>
-      <c r="C84" t="s">
-        <v>104</v>
-      </c>
-      <c r="D84">
-        <v>619</v>
-      </c>
-      <c r="E84" t="s">
-        <v>150</v>
-      </c>
-      <c r="F84">
-        <v>63</v>
-      </c>
-      <c r="G84" t="s">
-        <v>175</v>
-      </c>
-      <c r="H84">
-        <v>0</v>
-      </c>
-      <c r="I84">
-        <v>219062482434</v>
-      </c>
-      <c r="J84" t="s">
-        <v>239</v>
-      </c>
-      <c r="K84" t="s">
-        <v>152</v>
-      </c>
-      <c r="L84" t="s">
-        <v>152</v>
-      </c>
-      <c r="M84" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="85" spans="1:13">
-      <c r="A85" t="s">
-        <v>18</v>
-      </c>
-      <c r="B85" t="s">
-        <v>102</v>
-      </c>
-      <c r="C85" t="s">
-        <v>104</v>
-      </c>
-      <c r="D85">
-        <v>2716</v>
-      </c>
-      <c r="E85" t="s">
-        <v>151</v>
-      </c>
-      <c r="F85">
-        <v>0</v>
-      </c>
-      <c r="G85" t="s">
-        <v>114</v>
-      </c>
-      <c r="H85">
-        <v>10</v>
-      </c>
-      <c r="I85">
-        <v>17191106</v>
-      </c>
-      <c r="J85" t="s">
-        <v>240</v>
-      </c>
-      <c r="K85" t="s">
-        <v>152</v>
-      </c>
-      <c r="L85" t="s">
-        <v>152</v>
-      </c>
-      <c r="M85" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="86" spans="1:13">
-      <c r="A86" t="s">
-        <v>18</v>
-      </c>
-      <c r="B86" t="s">
-        <v>103</v>
-      </c>
-      <c r="C86" t="s">
-        <v>104</v>
-      </c>
-      <c r="D86">
-        <v>2716</v>
-      </c>
-      <c r="E86" t="s">
-        <v>151</v>
-      </c>
-      <c r="F86">
-        <v>0</v>
-      </c>
-      <c r="G86" t="s">
-        <v>114</v>
-      </c>
-      <c r="H86">
-        <v>64</v>
-      </c>
-      <c r="I86">
-        <v>1456427251</v>
-      </c>
-      <c r="J86" t="s">
-        <v>241</v>
-      </c>
-      <c r="K86" t="s">
-        <v>152</v>
-      </c>
-      <c r="L86" t="s">
-        <v>152</v>
-      </c>
-      <c r="M86" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fin eda 1 inicio eda 2
</commit_message>
<xml_diff>
--- a/Reporte_Estructura_Dataset.xlsx
+++ b/Reporte_Estructura_Dataset.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="239">
   <si>
     <t>Grupo</t>
   </si>
@@ -259,6 +259,9 @@
     <t>sp_editorial_playlist_total_reach</t>
   </si>
   <si>
+    <t>sp_playlist_total_reach</t>
+  </si>
+  <si>
     <t>yt_playlist_total_reach</t>
   </si>
   <si>
@@ -301,9 +304,6 @@
     <t>sp_monthly_listeners</t>
   </si>
   <si>
-    <t>sp_playlist_total_reach</t>
-  </si>
-  <si>
     <t>sp_popularity</t>
   </si>
   <si>
@@ -331,9 +331,6 @@
     <t>bool</t>
   </si>
   <si>
-    <t>str</t>
-  </si>
-  <si>
     <t>boolean</t>
   </si>
   <si>
@@ -520,18 +517,6 @@
     <t>0.90%</t>
   </si>
   <si>
-    <t>'s-Hertogenbosch</t>
-  </si>
-  <si>
-    <t>$NOT</t>
-  </si>
-  <si>
-    <t>Żelazowa Wola</t>
-  </si>
-  <si>
-    <t>酷狗文化</t>
-  </si>
-  <si>
     <t>1450.44</t>
   </si>
   <si>
@@ -670,6 +655,9 @@
     <t>15862733.71</t>
   </si>
   <si>
+    <t>54687523.16</t>
+  </si>
+  <si>
     <t>382175962.73</t>
   </si>
   <si>
@@ -710,9 +698,6 @@
   </si>
   <si>
     <t>6011495.49</t>
-  </si>
-  <si>
-    <t>54687523.16</t>
   </si>
   <si>
     <t>60.38</t>
@@ -1168,13 +1153,13 @@
         <v>5002</v>
       </c>
       <c r="E2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H2">
         <v>9</v>
@@ -1183,16 +1168,16 @@
         <v>66275</v>
       </c>
       <c r="J2" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="K2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1209,13 +1194,13 @@
         <v>4579</v>
       </c>
       <c r="E3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H3">
         <v>20</v>
@@ -1224,16 +1209,16 @@
         <v>50153</v>
       </c>
       <c r="J3" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="K3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1250,13 +1235,13 @@
         <v>5002</v>
       </c>
       <c r="E4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -1265,16 +1250,16 @@
         <v>1498</v>
       </c>
       <c r="J4" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="K4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1291,13 +1276,13 @@
         <v>4579</v>
       </c>
       <c r="E5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1306,16 +1291,16 @@
         <v>22055</v>
       </c>
       <c r="J5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="K5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1332,13 +1317,13 @@
         <v>4005</v>
       </c>
       <c r="E6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H6">
         <v>60</v>
@@ -1347,16 +1332,16 @@
         <v>90000</v>
       </c>
       <c r="J6" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="K6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1373,13 +1358,13 @@
         <v>3526</v>
       </c>
       <c r="E7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1388,16 +1373,16 @@
         <v>250000</v>
       </c>
       <c r="J7" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="K7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1414,13 +1399,13 @@
         <v>3130</v>
       </c>
       <c r="E8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H8">
         <v>75</v>
@@ -1429,16 +1414,16 @@
         <v>130975</v>
       </c>
       <c r="J8" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="K8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1455,31 +1440,31 @@
         <v>4733</v>
       </c>
       <c r="E9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K9">
         <v>14</v>
       </c>
       <c r="L9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1496,31 +1481,31 @@
         <v>4375</v>
       </c>
       <c r="E10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K10">
         <v>14</v>
       </c>
       <c r="L10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1537,13 +1522,13 @@
         <v>3816</v>
       </c>
       <c r="E11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F11">
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -1552,16 +1537,16 @@
         <v>84</v>
       </c>
       <c r="J11" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="K11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -1578,13 +1563,13 @@
         <v>3375</v>
       </c>
       <c r="E12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
       <c r="G12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -1593,16 +1578,16 @@
         <v>99</v>
       </c>
       <c r="J12" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="K12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1619,13 +1604,13 @@
         <v>2947</v>
       </c>
       <c r="E13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F13">
         <v>28</v>
       </c>
       <c r="G13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -1634,16 +1619,16 @@
         <v>140</v>
       </c>
       <c r="J13" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1660,13 +1645,13 @@
         <v>3816</v>
       </c>
       <c r="E14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F14">
         <v>0</v>
       </c>
       <c r="G14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -1675,16 +1660,16 @@
         <v>26</v>
       </c>
       <c r="J14" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="K14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -1701,13 +1686,13 @@
         <v>3375</v>
       </c>
       <c r="E15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F15">
         <v>0</v>
       </c>
       <c r="G15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -1716,16 +1701,16 @@
         <v>28</v>
       </c>
       <c r="J15" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="K15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -1742,13 +1727,13 @@
         <v>2947</v>
       </c>
       <c r="E16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F16">
         <v>28</v>
       </c>
       <c r="G16" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -1757,16 +1742,16 @@
         <v>31</v>
       </c>
       <c r="J16" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="K16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1783,13 +1768,13 @@
         <v>4733</v>
       </c>
       <c r="E17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F17">
         <v>0</v>
       </c>
       <c r="G17" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H17">
         <v>1</v>
@@ -1798,16 +1783,16 @@
         <v>8</v>
       </c>
       <c r="J17" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="K17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1824,13 +1809,13 @@
         <v>4375</v>
       </c>
       <c r="E18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
       <c r="G18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -1839,16 +1824,16 @@
         <v>10</v>
       </c>
       <c r="J18" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="K18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -1865,13 +1850,13 @@
         <v>3788</v>
       </c>
       <c r="E19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H19">
         <v>1</v>
@@ -1880,16 +1865,16 @@
         <v>90</v>
       </c>
       <c r="J19" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="K19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1906,13 +1891,13 @@
         <v>3321</v>
       </c>
       <c r="E20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
       <c r="G20" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -1921,16 +1906,16 @@
         <v>129</v>
       </c>
       <c r="J20" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="K20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -1947,13 +1932,13 @@
         <v>6777</v>
       </c>
       <c r="E21" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F21">
         <v>0</v>
       </c>
       <c r="G21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H21">
         <v>1</v>
@@ -1962,16 +1947,16 @@
         <v>118</v>
       </c>
       <c r="J21" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="K21" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L21" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M21" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -1988,13 +1973,13 @@
         <v>2087</v>
       </c>
       <c r="E22" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F22">
         <v>860</v>
       </c>
       <c r="G22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -2003,16 +1988,16 @@
         <v>179</v>
       </c>
       <c r="J22" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="K22" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L22" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M22" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -2029,13 +2014,13 @@
         <v>4005</v>
       </c>
       <c r="E23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F23">
         <v>0</v>
       </c>
       <c r="G23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H23">
         <v>1</v>
@@ -2044,16 +2029,16 @@
         <v>86</v>
       </c>
       <c r="J23" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="K23" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L23" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M23" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -2070,13 +2055,13 @@
         <v>3526</v>
       </c>
       <c r="E24" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F24">
         <v>0</v>
       </c>
       <c r="G24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H24">
         <v>1</v>
@@ -2085,16 +2070,16 @@
         <v>112</v>
       </c>
       <c r="J24" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="K24" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L24" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M24" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -2111,13 +2096,13 @@
         <v>2947</v>
       </c>
       <c r="E25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F25">
         <v>183</v>
       </c>
       <c r="G25" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -2126,16 +2111,16 @@
         <v>160</v>
       </c>
       <c r="J25" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K25" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L25" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M25" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -2152,13 +2137,13 @@
         <v>3816</v>
       </c>
       <c r="E26" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H26">
         <v>1</v>
@@ -2167,16 +2152,16 @@
         <v>72</v>
       </c>
       <c r="J26" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="K26" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L26" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M26" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -2193,13 +2178,13 @@
         <v>3375</v>
       </c>
       <c r="E27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F27">
         <v>0</v>
       </c>
       <c r="G27" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H27">
         <v>1</v>
@@ -2208,16 +2193,16 @@
         <v>129</v>
       </c>
       <c r="J27" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="K27" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L27" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M27" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -2234,13 +2219,13 @@
         <v>2975</v>
       </c>
       <c r="E28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F28">
         <v>0</v>
       </c>
       <c r="G28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H28">
         <v>1</v>
@@ -2249,16 +2234,16 @@
         <v>170</v>
       </c>
       <c r="J28" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="K28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -2275,13 +2260,13 @@
         <v>4005</v>
       </c>
       <c r="E29" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
       <c r="G29" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H29">
         <v>60</v>
@@ -2290,16 +2275,16 @@
         <v>3185238</v>
       </c>
       <c r="J29" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="K29" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L29" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M29" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -2316,13 +2301,13 @@
         <v>3526</v>
       </c>
       <c r="E30" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F30">
         <v>1</v>
       </c>
       <c r="G30" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H30">
         <v>0</v>
@@ -2331,16 +2316,16 @@
         <v>3350782</v>
       </c>
       <c r="J30" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="K30" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L30" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M30" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -2357,13 +2342,13 @@
         <v>3130</v>
       </c>
       <c r="E31" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H31">
         <v>75</v>
@@ -2372,16 +2357,16 @@
         <v>4167910</v>
       </c>
       <c r="J31" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="K31" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L31" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M31" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -2398,31 +2383,31 @@
         <v>0</v>
       </c>
       <c r="E32" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F32">
         <v>4980</v>
       </c>
       <c r="G32" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H32" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I32" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J32" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K32" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L32" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="M32" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
     </row>
     <row r="33" spans="1:13">
@@ -2439,31 +2424,31 @@
         <v>0</v>
       </c>
       <c r="E33" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F33" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G33" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H33" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I33" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J33" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K33">
         <v>5</v>
       </c>
       <c r="L33" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M33" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -2480,13 +2465,13 @@
         <v>0</v>
       </c>
       <c r="E34" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F34">
         <v>372</v>
       </c>
       <c r="G34" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H34">
         <v>0</v>
@@ -2495,16 +2480,16 @@
         <v>100</v>
       </c>
       <c r="J34" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="K34" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L34" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M34" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -2521,31 +2506,31 @@
         <v>0</v>
       </c>
       <c r="E35" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F35" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G35" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H35" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I35" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J35" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K35">
         <v>5</v>
       </c>
       <c r="L35" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M35" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -2562,13 +2547,13 @@
         <v>0</v>
       </c>
       <c r="E36" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F36">
         <v>82</v>
       </c>
       <c r="G36" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H36">
         <v>0</v>
@@ -2577,16 +2562,16 @@
         <v>100</v>
       </c>
       <c r="J36" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="K36" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L36" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M36" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -2603,13 +2588,13 @@
         <v>0</v>
       </c>
       <c r="E37" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F37">
         <v>0</v>
       </c>
       <c r="G37" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H37">
         <v>2</v>
@@ -2618,16 +2603,16 @@
         <v>14847778</v>
       </c>
       <c r="J37" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="K37" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L37" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M37" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -2644,13 +2629,13 @@
         <v>0</v>
       </c>
       <c r="E38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F38">
         <v>0</v>
       </c>
       <c r="G38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H38">
         <v>1</v>
@@ -2659,16 +2644,16 @@
         <v>458903</v>
       </c>
       <c r="J38" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="K38" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L38" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M38" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -2685,13 +2670,13 @@
         <v>0</v>
       </c>
       <c r="E39" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F39">
         <v>0</v>
       </c>
       <c r="G39" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H39">
         <v>26.02413665904167</v>
@@ -2700,16 +2685,16 @@
         <v>99.38711679376492</v>
       </c>
       <c r="J39" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="K39" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L39" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M39" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="40" spans="1:13">
@@ -2726,31 +2711,31 @@
         <v>67</v>
       </c>
       <c r="E40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F40" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G40" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H40" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I40" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J40" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K40">
         <v>112</v>
       </c>
       <c r="L40" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M40" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -2767,31 +2752,31 @@
         <v>67</v>
       </c>
       <c r="E41" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F41" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G41" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H41" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I41" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J41" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K41">
         <v>6</v>
       </c>
       <c r="L41" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M41" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -2808,31 +2793,31 @@
         <v>4561</v>
       </c>
       <c r="E42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K42">
         <v>11</v>
       </c>
       <c r="L42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -2849,31 +2834,31 @@
         <v>0</v>
       </c>
       <c r="E43" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F43" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G43" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H43" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I43" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J43" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K43">
         <v>12</v>
       </c>
       <c r="L43" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M43" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -2884,37 +2869,37 @@
         <v>61</v>
       </c>
       <c r="C44" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D44">
         <v>2608</v>
       </c>
       <c r="E44" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H44" t="s">
-        <v>168</v>
+        <v>145</v>
       </c>
       <c r="I44" t="s">
-        <v>170</v>
+        <v>145</v>
       </c>
       <c r="J44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K44">
         <v>1083</v>
       </c>
       <c r="L44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -2925,37 +2910,37 @@
         <v>62</v>
       </c>
       <c r="C45" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D45">
         <v>524</v>
       </c>
       <c r="E45" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F45">
         <v>4765</v>
       </c>
       <c r="G45" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L45" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="M45" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
     </row>
     <row r="46" spans="1:13">
@@ -2966,37 +2951,37 @@
         <v>63</v>
       </c>
       <c r="C46" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D46">
         <v>2310</v>
       </c>
       <c r="E46" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F46">
         <v>4053</v>
       </c>
       <c r="G46" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H46" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I46" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J46" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K46" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L46" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M46" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -3013,31 +2998,31 @@
         <v>0</v>
       </c>
       <c r="E47" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F47" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G47" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H47" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I47" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J47" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K47">
         <v>339</v>
       </c>
       <c r="L47" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M47" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -3054,31 +3039,31 @@
         <v>0</v>
       </c>
       <c r="E48" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F48" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G48" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H48" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I48" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J48" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K48">
         <v>4</v>
       </c>
       <c r="L48" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M48" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -3095,31 +3080,31 @@
         <v>0</v>
       </c>
       <c r="E49" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K49">
         <v>11</v>
       </c>
       <c r="L49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M49" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -3130,37 +3115,37 @@
         <v>67</v>
       </c>
       <c r="C50" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D50">
         <v>524</v>
       </c>
       <c r="E50" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F50" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G50" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H50" t="s">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="I50" t="s">
-        <v>171</v>
+        <v>145</v>
       </c>
       <c r="J50" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K50">
         <v>3574</v>
       </c>
       <c r="L50" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M50" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -3177,13 +3162,13 @@
         <v>543</v>
       </c>
       <c r="E51" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F51">
         <v>648</v>
       </c>
       <c r="G51" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H51">
         <v>0</v>
@@ -3192,16 +3177,16 @@
         <v>43152895</v>
       </c>
       <c r="J51" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="K51" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L51" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M51" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -3218,13 +3203,13 @@
         <v>543</v>
       </c>
       <c r="E52" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F52">
         <v>4</v>
       </c>
       <c r="G52" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H52">
         <v>0</v>
@@ -3233,16 +3218,16 @@
         <v>75271226</v>
       </c>
       <c r="J52" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="K52" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L52" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M52" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -3259,13 +3244,13 @@
         <v>226</v>
       </c>
       <c r="E53" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F53">
         <v>110</v>
       </c>
       <c r="G53" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H53">
         <v>0</v>
@@ -3274,16 +3259,16 @@
         <v>2473</v>
       </c>
       <c r="J53" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="K53" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L53" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M53" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -3300,13 +3285,13 @@
         <v>226</v>
       </c>
       <c r="E54" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F54">
         <v>0</v>
       </c>
       <c r="G54" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H54">
         <v>1</v>
@@ -3315,16 +3300,16 @@
         <v>6407</v>
       </c>
       <c r="J54" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="K54" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L54" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M54" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -3341,13 +3326,13 @@
         <v>799</v>
       </c>
       <c r="E55" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F55">
         <v>20</v>
       </c>
       <c r="G55" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H55">
         <v>0</v>
@@ -3356,16 +3341,16 @@
         <v>1570</v>
       </c>
       <c r="J55" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="K55" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L55" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M55" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -3382,13 +3367,13 @@
         <v>799</v>
       </c>
       <c r="E56" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F56">
         <v>0</v>
       </c>
       <c r="G56" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H56">
         <v>1</v>
@@ -3397,16 +3382,16 @@
         <v>1680</v>
       </c>
       <c r="J56" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="K56" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L56" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M56" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -3423,13 +3408,13 @@
         <v>543</v>
       </c>
       <c r="E57" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F57">
         <v>648</v>
       </c>
       <c r="G57" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H57">
         <v>0</v>
@@ -3438,16 +3423,16 @@
         <v>413</v>
       </c>
       <c r="J57" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K57" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L57" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M57" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -3464,13 +3449,13 @@
         <v>543</v>
       </c>
       <c r="E58" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F58">
         <v>0</v>
       </c>
       <c r="G58" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H58">
         <v>1</v>
@@ -3479,16 +3464,16 @@
         <v>2024</v>
       </c>
       <c r="J58" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="K58" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L58" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M58" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -3505,13 +3490,13 @@
         <v>11</v>
       </c>
       <c r="E59" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F59">
         <v>218</v>
       </c>
       <c r="G59" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H59">
         <v>0</v>
@@ -3520,16 +3505,16 @@
         <v>2393</v>
       </c>
       <c r="J59" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="K59" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L59" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M59" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -3546,13 +3531,13 @@
         <v>11</v>
       </c>
       <c r="E60" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F60">
         <v>0</v>
       </c>
       <c r="G60" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H60">
         <v>2</v>
@@ -3561,16 +3546,16 @@
         <v>3376367</v>
       </c>
       <c r="J60" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="K60" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L60" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M60" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -3587,13 +3572,13 @@
         <v>431</v>
       </c>
       <c r="E61" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F61">
         <v>703</v>
       </c>
       <c r="G61" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H61">
         <v>0</v>
@@ -3602,16 +3587,16 @@
         <v>204</v>
       </c>
       <c r="J61" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="K61" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L61" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M61" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -3628,13 +3613,13 @@
         <v>431</v>
       </c>
       <c r="E62" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F62">
         <v>0</v>
       </c>
       <c r="G62" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H62">
         <v>1</v>
@@ -3643,16 +3628,16 @@
         <v>1271</v>
       </c>
       <c r="J62" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K62" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L62" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M62" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="63" spans="1:13">
@@ -3669,13 +3654,13 @@
         <v>11</v>
       </c>
       <c r="E63" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F63">
         <v>244</v>
       </c>
       <c r="G63" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H63">
         <v>0</v>
@@ -3684,16 +3669,16 @@
         <v>401578965</v>
       </c>
       <c r="J63" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="K63" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L63" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M63" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -3707,75 +3692,75 @@
         <v>101</v>
       </c>
       <c r="D64">
-        <v>549</v>
+        <v>11</v>
       </c>
       <c r="E64" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="F64">
         <v>0</v>
       </c>
       <c r="G64" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H64">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I64">
-        <v>14446891354</v>
+        <v>1048509088</v>
       </c>
       <c r="J64" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="K64" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L64" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M64" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="65" spans="1:13">
       <c r="A65" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B65" t="s">
         <v>82</v>
       </c>
       <c r="C65" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D65">
-        <v>606</v>
+        <v>549</v>
       </c>
       <c r="E65" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F65">
         <v>0</v>
       </c>
       <c r="G65" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H65">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I65">
-        <v>415101450</v>
+        <v>14446891354</v>
       </c>
       <c r="J65" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="K65" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L65" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M65" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -3789,34 +3774,34 @@
         <v>103</v>
       </c>
       <c r="D66">
-        <v>2199</v>
+        <v>606</v>
       </c>
       <c r="E66" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F66">
         <v>0</v>
       </c>
       <c r="G66" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H66">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I66">
-        <v>92600000</v>
+        <v>415101450</v>
       </c>
       <c r="J66" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="K66" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L66" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M66" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="67" spans="1:13">
@@ -3833,31 +3818,31 @@
         <v>2199</v>
       </c>
       <c r="E67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F67">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="G67" t="s">
-        <v>163</v>
+        <v>121</v>
       </c>
       <c r="H67">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I67">
-        <v>5300000000</v>
+        <v>92600000</v>
       </c>
       <c r="J67" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="K67" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L67" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M67" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -3868,37 +3853,37 @@
         <v>85</v>
       </c>
       <c r="C68" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D68">
-        <v>66</v>
+        <v>2199</v>
       </c>
       <c r="E68" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F68">
-        <v>3</v>
+        <v>71</v>
       </c>
       <c r="G68" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H68">
         <v>0</v>
       </c>
       <c r="I68">
-        <v>294275870</v>
+        <v>5300000000</v>
       </c>
       <c r="J68" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="K68" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L68" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M68" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="69" spans="1:13">
@@ -3915,31 +3900,31 @@
         <v>66</v>
       </c>
       <c r="E69" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F69">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G69" t="s">
-        <v>122</v>
+        <v>163</v>
       </c>
       <c r="H69">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="I69">
-        <v>225624671689</v>
+        <v>294275870</v>
       </c>
       <c r="J69" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="K69" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L69" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M69" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="70" spans="1:13">
@@ -3953,34 +3938,34 @@
         <v>101</v>
       </c>
       <c r="D70">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E70" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="F70">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G70" t="s">
-        <v>164</v>
+        <v>121</v>
       </c>
       <c r="H70">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="I70">
-        <v>151680251</v>
+        <v>225624671689</v>
       </c>
       <c r="J70" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="K70" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L70" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M70" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="71" spans="1:13">
@@ -3991,42 +3976,42 @@
         <v>88</v>
       </c>
       <c r="C71" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D71">
-        <v>1773</v>
+        <v>67</v>
       </c>
       <c r="E71" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="F71">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G71" t="s">
-        <v>122</v>
+        <v>163</v>
       </c>
       <c r="H71">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I71">
-        <v>96700769</v>
+        <v>151680251</v>
       </c>
       <c r="J71" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="K71" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L71" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M71" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="72" spans="1:13">
       <c r="A72" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B72" t="s">
         <v>89</v>
@@ -4035,34 +4020,34 @@
         <v>103</v>
       </c>
       <c r="D72">
-        <v>198</v>
+        <v>1773</v>
       </c>
       <c r="E72" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F72">
         <v>0</v>
       </c>
       <c r="G72" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H72">
         <v>1</v>
       </c>
       <c r="I72">
-        <v>20740405</v>
+        <v>96700769</v>
       </c>
       <c r="J72" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="K72" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L72" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M72" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="73" spans="1:13">
@@ -4076,34 +4061,34 @@
         <v>103</v>
       </c>
       <c r="D73">
-        <v>670</v>
+        <v>198</v>
       </c>
       <c r="E73" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F73">
         <v>0</v>
       </c>
       <c r="G73" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H73">
         <v>1</v>
       </c>
       <c r="I73">
-        <v>92298921</v>
+        <v>20740405</v>
       </c>
       <c r="J73" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="K73" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L73" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M73" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="74" spans="1:13">
@@ -4117,34 +4102,34 @@
         <v>103</v>
       </c>
       <c r="D74">
-        <v>470</v>
+        <v>670</v>
       </c>
       <c r="E74" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F74">
         <v>0</v>
       </c>
       <c r="G74" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H74">
         <v>1</v>
       </c>
       <c r="I74">
-        <v>33495855298</v>
+        <v>92298921</v>
       </c>
       <c r="J74" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="K74" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L74" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M74" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="75" spans="1:13">
@@ -4158,34 +4143,34 @@
         <v>103</v>
       </c>
       <c r="D75">
-        <v>17</v>
+        <v>470</v>
       </c>
       <c r="E75" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F75">
         <v>0</v>
       </c>
       <c r="G75" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H75">
         <v>1</v>
       </c>
       <c r="I75">
-        <v>556229266</v>
+        <v>33495855298</v>
       </c>
       <c r="J75" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="K75" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L75" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M75" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="76" spans="1:13">
@@ -4199,34 +4184,34 @@
         <v>103</v>
       </c>
       <c r="D76">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E76" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F76">
         <v>0</v>
       </c>
       <c r="G76" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H76">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="I76">
-        <v>176892662</v>
+        <v>556229266</v>
       </c>
       <c r="J76" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="K76" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L76" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M76" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="77" spans="1:13">
@@ -4243,31 +4228,31 @@
         <v>22</v>
       </c>
       <c r="E77" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F77">
         <v>0</v>
       </c>
       <c r="G77" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H77">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I77">
-        <v>134166866</v>
+        <v>176892662</v>
       </c>
       <c r="J77" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="K77" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L77" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M77" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -4278,37 +4263,37 @@
         <v>95</v>
       </c>
       <c r="C78" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D78">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E78" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="F78">
         <v>0</v>
       </c>
       <c r="G78" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I78">
-        <v>1048509088</v>
+        <v>134166866</v>
       </c>
       <c r="J78" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="K78" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L78" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M78" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="79" spans="1:13">
@@ -4325,13 +4310,13 @@
         <v>8</v>
       </c>
       <c r="E79" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F79">
         <v>49</v>
       </c>
       <c r="G79" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H79">
         <v>0</v>
@@ -4340,16 +4325,16 @@
         <v>100</v>
       </c>
       <c r="J79" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="K79" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L79" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M79" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="80" spans="1:13">
@@ -4366,13 +4351,13 @@
         <v>619</v>
       </c>
       <c r="E80" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F80">
         <v>35</v>
       </c>
       <c r="G80" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H80">
         <v>0</v>
@@ -4381,16 +4366,16 @@
         <v>200000000</v>
       </c>
       <c r="J80" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="K80" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L80" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M80" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="81" spans="1:13">
@@ -4407,13 +4392,13 @@
         <v>619</v>
       </c>
       <c r="E81" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F81">
         <v>63</v>
       </c>
       <c r="G81" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H81">
         <v>0</v>
@@ -4422,16 +4407,16 @@
         <v>219062482434</v>
       </c>
       <c r="J81" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="K81" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L81" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M81" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="82" spans="1:13">
@@ -4448,13 +4433,13 @@
         <v>2716</v>
       </c>
       <c r="E82" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F82">
         <v>0</v>
       </c>
       <c r="G82" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H82">
         <v>10</v>
@@ -4463,16 +4448,16 @@
         <v>17191106</v>
       </c>
       <c r="J82" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="K82" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L82" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M82" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="83" spans="1:13">
@@ -4489,13 +4474,13 @@
         <v>2716</v>
       </c>
       <c r="E83" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F83">
         <v>0</v>
       </c>
       <c r="G83" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H83">
         <v>64</v>
@@ -4504,16 +4489,16 @@
         <v>1456427251</v>
       </c>
       <c r="J83" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="K83" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L83" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M83" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>